<commit_message>
Update pest data from SharePoint
</commit_message>
<xml_diff>
--- a/data.xlsx
+++ b/data.xlsx
@@ -3,9 +3,14 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
   <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30219"/>
   <workbookPr/>
-  <xr:revisionPtr revIDLastSave="1" documentId="11_BDD78AAB8A0CBC1AA983446414CCFA72D025956C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{3D66B755-C672-4EF6-B867-ACEFA14B501C}"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://wastea.sharepoint.com/sites/FourSeasonsPestIssues/Shared Documents/"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="77" documentId="11_BDD78AAB8A0CBC1AA983446414CCFA72D025956C" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{5EB0F648-B7F8-4F5B-A8FB-07F528ECC564}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="0" windowHeight="0" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-48" yWindow="-48" windowWidth="23136" windowHeight="12336" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Glitches" sheetId="1" r:id="rId1"/>
@@ -32,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="104" uniqueCount="69">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="118" uniqueCount="74">
   <si>
     <t>ID</t>
   </si>
@@ -182,6 +187,21 @@
   </si>
   <si>
     <t>Rats in the kitchen store</t>
+  </si>
+  <si>
+    <t>G-022</t>
+  </si>
+  <si>
+    <t>29/06/2026</t>
+  </si>
+  <si>
+    <t>Rabbit eating carrots TEST123</t>
+  </si>
+  <si>
+    <t>G-011</t>
+  </si>
+  <si>
+    <t>Rabbit on the guest piullow</t>
   </si>
   <si>
     <t>Glitches / Pest Issues - Shared Workbook (SharePoint)</t>
@@ -246,7 +266,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="dd/mm/yyyy"/>
+    <numFmt numFmtId="164" formatCode="dd/mm/yyyy"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -273,7 +293,7 @@
       <name val="Arial"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -287,12 +307,30 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFEAF3EF"/>
+        <fgColor rgb="FFFFF6D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFFF6D6"/>
+        <fgColor theme="0"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="5" tint="0.79998168889431442"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
+        <bgColor theme="0" tint="-0.14999847407452621"/>
       </patternFill>
     </fill>
   </fills>
@@ -306,16 +344,16 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="FFC9D9D2"/>
+        <color indexed="64"/>
       </left>
       <right style="thin">
-        <color rgb="FFC9D9D2"/>
+        <color indexed="64"/>
       </right>
       <top style="thin">
-        <color rgb="FFC9D9D2"/>
+        <color indexed="64"/>
       </top>
       <bottom style="thin">
-        <color rgb="FFC9D9D2"/>
+        <color indexed="64"/>
       </bottom>
       <diagonal/>
     </border>
@@ -323,24 +361,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="2" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -348,6 +371,39 @@
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="4" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="2" fillId="6" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -651,395 +707,766 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:K11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:K37"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="1" max="1" width="9" customWidth="1"/>
-    <col min="2" max="2" width="12" customWidth="1"/>
-    <col min="3" max="3" width="11" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="22" customWidth="1"/>
-    <col min="6" max="6" width="34" customWidth="1"/>
-    <col min="7" max="7" width="10" customWidth="1"/>
-    <col min="8" max="8" width="13" customWidth="1"/>
-    <col min="9" max="9" width="38" customWidth="1"/>
-    <col min="10" max="10" width="13" customWidth="1"/>
-    <col min="11" max="11" width="14" customWidth="1"/>
+    <col min="1" max="1" width="9" style="15" customWidth="1"/>
+    <col min="2" max="2" width="12" style="16" customWidth="1"/>
+    <col min="3" max="3" width="14.28515625" style="15" customWidth="1"/>
+    <col min="4" max="4" width="17" style="15" customWidth="1"/>
+    <col min="5" max="5" width="22" style="15" customWidth="1"/>
+    <col min="6" max="6" width="34" style="15" customWidth="1"/>
+    <col min="7" max="7" width="12.42578125" style="15" customWidth="1"/>
+    <col min="8" max="8" width="13" style="15" customWidth="1"/>
+    <col min="9" max="9" width="38" style="15" customWidth="1"/>
+    <col min="10" max="10" width="16.140625" style="15" customWidth="1"/>
+    <col min="11" max="11" width="14.140625" style="15" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="15"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="24" customHeight="1">
-      <c r="A1" s="1" t="s">
+      <c r="A1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" s="13" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" s="13" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" s="13" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" s="13" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" s="13" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" s="13" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" s="13" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" s="13" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
-      <c r="A2" s="2" t="s">
+    <row r="2" spans="1:11" ht="15">
+      <c r="A2" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="5">
         <v>46192</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="4">
         <v>410</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E2" s="2" t="s">
+      <c r="E2" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="F2" s="2" t="s">
+      <c r="F2" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="G2" s="2" t="s">
+      <c r="G2" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H2" s="2" t="s">
+      <c r="H2" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I2" s="2" t="s">
+      <c r="I2" s="4" t="s">
         <v>17</v>
       </c>
-      <c r="J2" s="3">
+      <c r="J2" s="6">
         <v>46193</v>
       </c>
-      <c r="K2" s="2" t="s">
+      <c r="K2" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
-      <c r="A3" s="4" t="s">
+    <row r="3" spans="1:11" ht="15">
+      <c r="A3" s="7" t="s">
         <v>19</v>
       </c>
-      <c r="B3" s="5">
+      <c r="B3" s="8">
         <v>46192</v>
       </c>
-      <c r="C3" s="4">
+      <c r="C3" s="7">
         <v>604</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="7" t="s">
         <v>20</v>
       </c>
-      <c r="F3" s="4" t="s">
+      <c r="F3" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="G3" s="4" t="s">
+      <c r="G3" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H3" s="4" t="s">
+      <c r="H3" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I3" s="4" t="s">
+      <c r="I3" s="7" t="s">
         <v>22</v>
       </c>
-      <c r="J3" s="5">
+      <c r="J3" s="9">
         <v>46192</v>
       </c>
-      <c r="K3" s="4" t="s">
+      <c r="K3" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
-      <c r="A4" s="2" t="s">
+    <row r="4" spans="1:11" ht="15">
+      <c r="A4" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="5">
         <v>46192</v>
       </c>
-      <c r="C4" s="2">
+      <c r="C4" s="4">
         <v>106</v>
       </c>
-      <c r="D4" s="2" t="s">
+      <c r="D4" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E4" s="2" t="s">
+      <c r="E4" s="4" t="s">
         <v>25</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G4" s="2" t="s">
+      <c r="G4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H4" s="2" t="s">
+      <c r="H4" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="I4" s="2" t="s">
+      <c r="I4" s="4" t="s">
         <v>27</v>
       </c>
-      <c r="J4" s="3">
+      <c r="J4" s="6">
         <v>46193</v>
       </c>
-      <c r="K4" s="2" t="s">
+      <c r="K4" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="5" spans="1:11">
-      <c r="A5" s="4" t="s">
+    <row r="5" spans="1:11" ht="15">
+      <c r="A5" s="7" t="s">
         <v>29</v>
       </c>
-      <c r="B5" s="5">
+      <c r="B5" s="8">
         <v>46193</v>
       </c>
-      <c r="C5" s="4">
+      <c r="C5" s="7">
         <v>604</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F5" s="4" t="s">
+      <c r="F5" s="7" t="s">
         <v>30</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="7" t="s">
         <v>15</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="I5" s="7" t="s">
         <v>31</v>
       </c>
-      <c r="J5" s="5">
+      <c r="J5" s="9">
         <v>46193</v>
       </c>
-      <c r="K5" s="4" t="s">
+      <c r="K5" s="7" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="6" spans="1:11">
-      <c r="A6" s="2" t="s">
+    <row r="6" spans="1:11" ht="15">
+      <c r="A6" s="4" t="s">
         <v>32</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="5">
         <v>46194</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="4">
         <v>112</v>
       </c>
-      <c r="D6" s="2" t="s">
+      <c r="D6" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E6" s="2" t="s">
+      <c r="E6" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="F6" s="2" t="s">
+      <c r="F6" s="4" t="s">
         <v>26</v>
       </c>
-      <c r="G6" s="2" t="s">
+      <c r="G6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="H6" s="2" t="s">
+      <c r="H6" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="I6" s="2" t="s">
+      <c r="I6" s="4" t="s">
         <v>34</v>
       </c>
-      <c r="J6" s="3">
+      <c r="J6" s="6">
         <v>46195</v>
       </c>
-      <c r="K6" s="2" t="s">
+      <c r="K6" s="4" t="s">
         <v>28</v>
       </c>
     </row>
-    <row r="7" spans="1:11">
-      <c r="A7" s="4" t="s">
+    <row r="7" spans="1:11" ht="15">
+      <c r="A7" s="7" t="s">
         <v>35</v>
       </c>
-      <c r="B7" s="5">
+      <c r="B7" s="8">
         <v>46194</v>
       </c>
-      <c r="C7" s="4">
+      <c r="C7" s="7">
         <v>104</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F7" s="4" t="s">
+      <c r="F7" s="7" t="s">
         <v>37</v>
       </c>
-      <c r="G7" s="4" t="s">
+      <c r="G7" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H7" s="4" t="s">
+      <c r="H7" s="7" t="s">
         <v>33</v>
       </c>
-      <c r="I7" s="4" t="s">
+      <c r="I7" s="7" t="s">
         <v>39</v>
       </c>
-      <c r="J7" s="5">
+      <c r="J7" s="9">
         <v>46195</v>
       </c>
-      <c r="K7" s="4" t="s">
+      <c r="K7" s="7" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:11">
-      <c r="A8" s="2" t="s">
+    <row r="8" spans="1:11" ht="15">
+      <c r="A8" s="4" t="s">
         <v>40</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="5">
         <v>46197</v>
       </c>
-      <c r="C8" s="2">
+      <c r="C8" s="4">
         <v>118</v>
       </c>
-      <c r="D8" s="2" t="s">
+      <c r="D8" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E8" s="2" t="s">
+      <c r="E8" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="4" t="s">
         <v>37</v>
       </c>
-      <c r="G8" s="2" t="s">
+      <c r="G8" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H8" s="2" t="s">
+      <c r="H8" s="4" t="s">
         <v>41</v>
       </c>
-      <c r="I8" s="2"/>
-      <c r="J8" s="3"/>
-      <c r="K8" s="2"/>
-    </row>
-    <row r="9" spans="1:11">
-      <c r="A9" s="4" t="s">
+      <c r="I8" s="4"/>
+      <c r="J8" s="6"/>
+      <c r="K8" s="4"/>
+    </row>
+    <row r="9" spans="1:11" ht="15">
+      <c r="A9" s="7" t="s">
         <v>42</v>
       </c>
-      <c r="B9" s="5">
+      <c r="B9" s="8">
         <v>46199</v>
       </c>
-      <c r="C9" s="4">
+      <c r="C9" s="7">
         <v>112</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="7" t="s">
         <v>13</v>
       </c>
-      <c r="F9" s="4" t="s">
+      <c r="F9" s="7" t="s">
         <v>43</v>
       </c>
-      <c r="G9" s="4" t="s">
+      <c r="G9" s="7" t="s">
         <v>44</v>
       </c>
-      <c r="H9" s="4" t="s">
+      <c r="H9" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="I9" s="4"/>
-      <c r="J9" s="5"/>
-      <c r="K9" s="4"/>
-    </row>
-    <row r="10" spans="1:11">
-      <c r="A10" s="2" t="s">
+      <c r="I9" s="7"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="7"/>
+    </row>
+    <row r="10" spans="1:11" ht="15">
+      <c r="A10" s="4" t="s">
         <v>45</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="5">
         <v>46196</v>
       </c>
-      <c r="C10" s="2">
+      <c r="C10" s="4">
         <v>210</v>
       </c>
-      <c r="D10" s="2" t="s">
+      <c r="D10" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E10" s="2" t="s">
+      <c r="E10" s="4" t="s">
         <v>36</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="4" t="s">
         <v>46</v>
       </c>
-      <c r="G10" s="2" t="s">
+      <c r="G10" s="4" t="s">
         <v>38</v>
       </c>
-      <c r="H10" s="2" t="s">
+      <c r="H10" s="4" t="s">
         <v>33</v>
       </c>
-      <c r="I10" s="2" t="s">
+      <c r="I10" s="4" t="s">
         <v>47</v>
       </c>
-      <c r="J10" s="3">
+      <c r="J10" s="6">
         <v>46197</v>
       </c>
-      <c r="K10" s="2" t="s">
+      <c r="K10" s="4" t="s">
         <v>18</v>
       </c>
     </row>
-    <row r="11" spans="1:11">
-      <c r="A11" s="4" t="s">
+    <row r="11" spans="1:11" ht="15">
+      <c r="A11" s="7" t="s">
         <v>48</v>
       </c>
       <c r="B11" s="5">
         <v>46198</v>
       </c>
-      <c r="C11" s="4">
+      <c r="C11" s="7">
         <v>305</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="7" t="s">
         <v>36</v>
       </c>
-      <c r="F11" s="4" t="s">
+      <c r="F11" s="7" t="s">
         <v>49</v>
       </c>
-      <c r="G11" s="4" t="s">
+      <c r="G11" s="7" t="s">
         <v>38</v>
       </c>
-      <c r="H11" s="4" t="s">
+      <c r="H11" s="7" t="s">
         <v>41</v>
       </c>
-      <c r="I11" s="4"/>
-      <c r="J11" s="5"/>
-      <c r="K11" s="4"/>
+      <c r="I11" s="7"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="7"/>
+    </row>
+    <row r="12" spans="1:11" ht="15">
+      <c r="A12" s="10" t="s">
+        <v>50</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C12" s="11">
+        <v>112</v>
+      </c>
+      <c r="D12" s="11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" s="11" t="s">
+        <v>36</v>
+      </c>
+      <c r="F12" s="11" t="s">
+        <v>52</v>
+      </c>
+      <c r="G12" s="11" t="s">
+        <v>44</v>
+      </c>
+      <c r="H12" s="11" t="s">
+        <v>33</v>
+      </c>
+      <c r="I12" s="11"/>
+      <c r="J12" s="11"/>
+      <c r="K12" s="11"/>
+    </row>
+    <row r="13" spans="1:11" ht="15">
+      <c r="A13" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="C13" s="12">
+        <v>111</v>
+      </c>
+      <c r="D13" s="12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" s="12" t="s">
+        <v>25</v>
+      </c>
+      <c r="F13" s="12" t="s">
+        <v>54</v>
+      </c>
+      <c r="G13" s="12" t="s">
+        <v>38</v>
+      </c>
+      <c r="H13" s="12" t="s">
+        <v>41</v>
+      </c>
+      <c r="I13" s="12"/>
+      <c r="J13" s="12"/>
+      <c r="K13" s="12"/>
+    </row>
+    <row r="14" spans="1:11" ht="15">
+      <c r="A14" s="10"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="11"/>
+      <c r="D14" s="11"/>
+      <c r="E14" s="11"/>
+      <c r="F14" s="11"/>
+      <c r="G14" s="11"/>
+      <c r="H14" s="11"/>
+      <c r="I14" s="11"/>
+      <c r="J14" s="11"/>
+      <c r="K14" s="11"/>
+    </row>
+    <row r="15" spans="1:11" ht="15">
+      <c r="A15" s="4"/>
+      <c r="B15" s="5"/>
+      <c r="C15" s="12"/>
+      <c r="D15" s="12"/>
+      <c r="E15" s="12"/>
+      <c r="F15" s="12"/>
+      <c r="G15" s="12"/>
+      <c r="H15" s="12"/>
+      <c r="I15" s="12"/>
+      <c r="J15" s="12"/>
+      <c r="K15" s="12"/>
+    </row>
+    <row r="16" spans="1:11" ht="15">
+      <c r="A16" s="10"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="11"/>
+      <c r="D16" s="11"/>
+      <c r="E16" s="11"/>
+      <c r="F16" s="11"/>
+      <c r="G16" s="11"/>
+      <c r="H16" s="11"/>
+      <c r="I16" s="11"/>
+      <c r="J16" s="11"/>
+      <c r="K16" s="11"/>
+    </row>
+    <row r="17" spans="1:11" ht="15">
+      <c r="A17" s="4"/>
+      <c r="B17" s="5"/>
+      <c r="C17" s="12"/>
+      <c r="D17" s="12"/>
+      <c r="E17" s="12"/>
+      <c r="F17" s="12"/>
+      <c r="G17" s="12"/>
+      <c r="H17" s="12"/>
+      <c r="I17" s="12"/>
+      <c r="J17" s="12"/>
+      <c r="K17" s="12"/>
+    </row>
+    <row r="18" spans="1:11" ht="15">
+      <c r="A18" s="10"/>
+      <c r="B18" s="5"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
+      <c r="I18" s="11"/>
+      <c r="J18" s="11"/>
+      <c r="K18" s="11"/>
+    </row>
+    <row r="19" spans="1:11" ht="15">
+      <c r="A19" s="4"/>
+      <c r="B19" s="5"/>
+      <c r="C19" s="12"/>
+      <c r="D19" s="12"/>
+      <c r="E19" s="12"/>
+      <c r="F19" s="12"/>
+      <c r="G19" s="12"/>
+      <c r="H19" s="12"/>
+      <c r="I19" s="12"/>
+      <c r="J19" s="12"/>
+      <c r="K19" s="12"/>
+    </row>
+    <row r="20" spans="1:11" ht="15">
+      <c r="A20" s="10"/>
+      <c r="B20" s="5"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
+      <c r="I20" s="11"/>
+      <c r="J20" s="11"/>
+      <c r="K20" s="11"/>
+    </row>
+    <row r="21" spans="1:11" ht="15">
+      <c r="A21" s="4"/>
+      <c r="B21" s="5"/>
+      <c r="C21" s="12"/>
+      <c r="D21" s="12"/>
+      <c r="E21" s="12"/>
+      <c r="F21" s="12"/>
+      <c r="G21" s="12"/>
+      <c r="H21" s="12"/>
+      <c r="I21" s="12"/>
+      <c r="J21" s="12"/>
+      <c r="K21" s="12"/>
+    </row>
+    <row r="22" spans="1:11" ht="15">
+      <c r="A22" s="10"/>
+      <c r="B22" s="5"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="11"/>
+      <c r="I22" s="11"/>
+      <c r="J22" s="11"/>
+      <c r="K22" s="11"/>
+    </row>
+    <row r="23" spans="1:11" ht="15">
+      <c r="A23" s="4"/>
+      <c r="B23" s="5"/>
+      <c r="C23" s="12"/>
+      <c r="D23" s="12"/>
+      <c r="E23" s="12"/>
+      <c r="F23" s="12"/>
+      <c r="G23" s="12"/>
+      <c r="H23" s="12"/>
+      <c r="I23" s="12"/>
+      <c r="J23" s="12"/>
+      <c r="K23" s="12"/>
+    </row>
+    <row r="24" spans="1:11" ht="15">
+      <c r="A24" s="10"/>
+      <c r="B24" s="5"/>
+      <c r="C24" s="11"/>
+      <c r="D24" s="11"/>
+      <c r="E24" s="11"/>
+      <c r="F24" s="11"/>
+      <c r="G24" s="11"/>
+      <c r="H24" s="11"/>
+      <c r="I24" s="11"/>
+      <c r="J24" s="11"/>
+      <c r="K24" s="11"/>
+    </row>
+    <row r="25" spans="1:11" ht="15">
+      <c r="A25" s="4"/>
+      <c r="B25" s="5"/>
+      <c r="C25" s="12"/>
+      <c r="D25" s="12"/>
+      <c r="E25" s="12"/>
+      <c r="F25" s="12"/>
+      <c r="G25" s="12"/>
+      <c r="H25" s="12"/>
+      <c r="I25" s="12"/>
+      <c r="J25" s="12"/>
+      <c r="K25" s="12"/>
+    </row>
+    <row r="26" spans="1:11" ht="15">
+      <c r="A26" s="10"/>
+      <c r="B26" s="5"/>
+      <c r="C26" s="11"/>
+      <c r="D26" s="11"/>
+      <c r="E26" s="11"/>
+      <c r="F26" s="11"/>
+      <c r="G26" s="11"/>
+      <c r="H26" s="11"/>
+      <c r="I26" s="11"/>
+      <c r="J26" s="11"/>
+      <c r="K26" s="11"/>
+    </row>
+    <row r="27" spans="1:11" ht="15">
+      <c r="A27" s="4"/>
+      <c r="B27" s="5"/>
+      <c r="C27" s="12"/>
+      <c r="D27" s="12"/>
+      <c r="E27" s="12"/>
+      <c r="F27" s="12"/>
+      <c r="G27" s="12"/>
+      <c r="H27" s="12"/>
+      <c r="I27" s="12"/>
+      <c r="J27" s="12"/>
+      <c r="K27" s="12"/>
+    </row>
+    <row r="28" spans="1:11" ht="15">
+      <c r="A28" s="10"/>
+      <c r="B28" s="5"/>
+      <c r="C28" s="11"/>
+      <c r="D28" s="11"/>
+      <c r="E28" s="11"/>
+      <c r="F28" s="11"/>
+      <c r="G28" s="11"/>
+      <c r="H28" s="11"/>
+      <c r="I28" s="11"/>
+      <c r="J28" s="11"/>
+      <c r="K28" s="11"/>
+    </row>
+    <row r="29" spans="1:11" ht="15">
+      <c r="A29" s="4"/>
+      <c r="B29" s="5"/>
+      <c r="C29" s="12"/>
+      <c r="D29" s="12"/>
+      <c r="E29" s="12"/>
+      <c r="F29" s="12"/>
+      <c r="G29" s="12"/>
+      <c r="H29" s="12"/>
+      <c r="I29" s="12"/>
+      <c r="J29" s="12"/>
+      <c r="K29" s="12"/>
+    </row>
+    <row r="30" spans="1:11" ht="15">
+      <c r="A30" s="10"/>
+      <c r="B30" s="5"/>
+      <c r="C30" s="11"/>
+      <c r="D30" s="11"/>
+      <c r="E30" s="11"/>
+      <c r="F30" s="11"/>
+      <c r="G30" s="11"/>
+      <c r="H30" s="11"/>
+      <c r="I30" s="11"/>
+      <c r="J30" s="11"/>
+      <c r="K30" s="11"/>
+    </row>
+    <row r="31" spans="1:11" ht="15">
+      <c r="A31" s="4"/>
+      <c r="B31" s="5"/>
+      <c r="C31" s="12"/>
+      <c r="D31" s="12"/>
+      <c r="E31" s="12"/>
+      <c r="F31" s="12"/>
+      <c r="G31" s="12"/>
+      <c r="H31" s="12"/>
+      <c r="I31" s="12"/>
+      <c r="J31" s="12"/>
+      <c r="K31" s="12"/>
+    </row>
+    <row r="32" spans="1:11" ht="15">
+      <c r="A32" s="10"/>
+      <c r="B32" s="5"/>
+      <c r="C32" s="11"/>
+      <c r="D32" s="11"/>
+      <c r="E32" s="11"/>
+      <c r="F32" s="11"/>
+      <c r="G32" s="11"/>
+      <c r="H32" s="11"/>
+      <c r="I32" s="11"/>
+      <c r="J32" s="11"/>
+      <c r="K32" s="11"/>
+    </row>
+    <row r="33" spans="1:11" ht="15">
+      <c r="A33" s="4"/>
+      <c r="B33" s="5"/>
+      <c r="C33" s="12"/>
+      <c r="D33" s="12"/>
+      <c r="E33" s="12"/>
+      <c r="F33" s="12"/>
+      <c r="G33" s="12"/>
+      <c r="H33" s="12"/>
+      <c r="I33" s="12"/>
+      <c r="J33" s="12"/>
+      <c r="K33" s="12"/>
+    </row>
+    <row r="34" spans="1:11" ht="15">
+      <c r="A34" s="10"/>
+      <c r="B34" s="5"/>
+      <c r="C34" s="11"/>
+      <c r="D34" s="11"/>
+      <c r="E34" s="11"/>
+      <c r="F34" s="11"/>
+      <c r="G34" s="11"/>
+      <c r="H34" s="11"/>
+      <c r="I34" s="11"/>
+      <c r="J34" s="11"/>
+      <c r="K34" s="11"/>
+    </row>
+    <row r="35" spans="1:11" ht="15">
+      <c r="A35" s="4"/>
+      <c r="B35" s="5"/>
+      <c r="C35" s="12"/>
+      <c r="D35" s="12"/>
+      <c r="E35" s="12"/>
+      <c r="F35" s="12"/>
+      <c r="G35" s="12"/>
+      <c r="H35" s="12"/>
+      <c r="I35" s="12"/>
+      <c r="J35" s="12"/>
+      <c r="K35" s="12"/>
+    </row>
+    <row r="36" spans="1:11" ht="15">
+      <c r="A36" s="10"/>
+      <c r="B36" s="5"/>
+      <c r="C36" s="11"/>
+      <c r="D36" s="11"/>
+      <c r="E36" s="11"/>
+      <c r="F36" s="11"/>
+      <c r="G36" s="11"/>
+      <c r="H36" s="11"/>
+      <c r="I36" s="11"/>
+      <c r="J36" s="11"/>
+      <c r="K36" s="11"/>
+    </row>
+    <row r="37" spans="1:11" ht="15">
+      <c r="A37" s="4"/>
+      <c r="B37" s="5"/>
+      <c r="C37" s="12"/>
+      <c r="D37" s="12"/>
+      <c r="E37" s="12"/>
+      <c r="F37" s="12"/>
+      <c r="G37" s="12"/>
+      <c r="H37" s="12"/>
+      <c r="I37" s="12"/>
+      <c r="J37" s="12"/>
+      <c r="K37" s="12"/>
     </row>
   </sheetData>
   <dataValidations count="2">
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list" sqref="G2:G500" xr:uid="{00000000-0002-0000-0000-000000000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list" sqref="G2:G489" xr:uid="{00000000-0002-0000-0000-000000000000}">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
-    <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list" sqref="H2:H500" xr:uid="{00000000-0002-0000-0000-000001000000}">
+    <dataValidation type="list" allowBlank="1" errorTitle="Invalid entry" error="Pick a value from the list" sqref="H2:H489" xr:uid="{00000000-0002-0000-0000-000001000000}">
       <formula1>"Open,In Progress,Resolved"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1050,119 +1477,119 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:A24"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="1" width="104" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="6" t="s">
-        <v>50</v>
+    <row r="1" spans="1:1" ht="15.6">
+      <c r="A1" s="1" t="s">
+        <v>55</v>
       </c>
     </row>
     <row r="2" spans="1:1">
-      <c r="A2" s="7"/>
+      <c r="A2" s="2"/>
     </row>
     <row r="3" spans="1:1">
-      <c r="A3" s="7" t="s">
-        <v>51</v>
+      <c r="A3" s="2" t="s">
+        <v>56</v>
       </c>
     </row>
     <row r="4" spans="1:1">
-      <c r="A4" s="7" t="s">
-        <v>52</v>
+      <c r="A4" s="2" t="s">
+        <v>57</v>
       </c>
     </row>
     <row r="5" spans="1:1">
-      <c r="A5" s="7"/>
-    </row>
-    <row r="6" spans="1:1">
-      <c r="A6" s="8" t="s">
-        <v>53</v>
+      <c r="A5" s="2"/>
+    </row>
+    <row r="6" spans="1:1" ht="15.6">
+      <c r="A6" s="3" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="7" spans="1:1">
-      <c r="A7" s="7" t="s">
-        <v>54</v>
+      <c r="A7" s="2" t="s">
+        <v>59</v>
       </c>
     </row>
     <row r="8" spans="1:1">
-      <c r="A8" s="7" t="s">
-        <v>55</v>
+      <c r="A8" s="2" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="9" spans="1:1">
-      <c r="A9" s="7" t="s">
-        <v>56</v>
+      <c r="A9" s="2" t="s">
+        <v>61</v>
       </c>
     </row>
     <row r="10" spans="1:1">
-      <c r="A10" s="7" t="s">
-        <v>57</v>
+      <c r="A10" s="2" t="s">
+        <v>62</v>
       </c>
     </row>
     <row r="11" spans="1:1">
-      <c r="A11" s="7" t="s">
-        <v>58</v>
+      <c r="A11" s="2" t="s">
+        <v>63</v>
       </c>
     </row>
     <row r="12" spans="1:1">
-      <c r="A12" s="7"/>
-    </row>
-    <row r="13" spans="1:1">
-      <c r="A13" s="8" t="s">
-        <v>59</v>
+      <c r="A12" s="2"/>
+    </row>
+    <row r="13" spans="1:1" ht="15.6">
+      <c r="A13" s="3" t="s">
+        <v>64</v>
       </c>
     </row>
     <row r="14" spans="1:1">
-      <c r="A14" s="7" t="s">
-        <v>60</v>
+      <c r="A14" s="2" t="s">
+        <v>65</v>
       </c>
     </row>
     <row r="15" spans="1:1">
-      <c r="A15" s="7" t="s">
-        <v>61</v>
+      <c r="A15" s="2" t="s">
+        <v>66</v>
       </c>
     </row>
     <row r="16" spans="1:1">
-      <c r="A16" s="7" t="s">
-        <v>62</v>
+      <c r="A16" s="2" t="s">
+        <v>67</v>
       </c>
     </row>
     <row r="17" spans="1:1">
-      <c r="A17" s="7" t="s">
-        <v>63</v>
+      <c r="A17" s="2" t="s">
+        <v>68</v>
       </c>
     </row>
     <row r="18" spans="1:1">
-      <c r="A18" s="7" t="s">
-        <v>64</v>
+      <c r="A18" s="2" t="s">
+        <v>69</v>
       </c>
     </row>
     <row r="19" spans="1:1">
-      <c r="A19" s="7" t="s">
-        <v>65</v>
+      <c r="A19" s="2" t="s">
+        <v>70</v>
       </c>
     </row>
     <row r="20" spans="1:1">
-      <c r="A20" s="7"/>
-    </row>
-    <row r="21" spans="1:1">
-      <c r="A21" s="8" t="s">
-        <v>66</v>
+      <c r="A20" s="2"/>
+    </row>
+    <row r="21" spans="1:1" ht="31.15">
+      <c r="A21" s="3" t="s">
+        <v>71</v>
       </c>
     </row>
     <row r="22" spans="1:1">
-      <c r="A22" s="7"/>
+      <c r="A22" s="2"/>
     </row>
     <row r="23" spans="1:1">
-      <c r="A23" s="7" t="s">
-        <v>67</v>
+      <c r="A23" s="2" t="s">
+        <v>72</v>
       </c>
     </row>
     <row r="24" spans="1:1">
-      <c r="A24" s="7" t="s">
-        <v>68</v>
+      <c r="A24" s="2" t="s">
+        <v>73</v>
       </c>
     </row>
   </sheetData>
@@ -1177,15 +1604,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010065EBA211F469494B95566F0690462C0F" ma:contentTypeVersion="3" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="b35d5fe4402d31ba90210c08896e5cda">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="09bf2ab9-8b38-4f4a-bdf8-acc823517723" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="f1cc7b22e06c9225b2664b95b39fc95f" ns2:_="">
     <xsd:import namespace="09bf2ab9-8b38-4f4a-bdf8-acc823517723"/>
@@ -1323,14 +1741,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{8501DBAD-27FE-47DE-8EC8-9F821B6253B3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{404E6A0B-DD94-4BD8-AF3F-E05CD29C39C9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{662F6FC7-D035-42E3-93B4-FE5EA88476C1}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{662F6FC7-D035-42E3-93B4-FE5EA88476C1}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{404E6A0B-DD94-4BD8-AF3F-E05CD29C39C9}"/>
 </file>
</xml_diff>